<commit_message>
fill in by period
</commit_message>
<xml_diff>
--- a/01-empty.xlsx
+++ b/01-empty.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="119">
   <si>
     <t>MINISTERIO DE EDUCACIÓN</t>
   </si>
@@ -135,10 +135,16 @@
     <t>lidada</t>
   </si>
   <si>
+    <t>aaaa</t>
+  </si>
+  <si>
     <t>AMAYA CASTRO, JIMENA GRISBEL</t>
   </si>
   <si>
     <t>F</t>
+  </si>
+  <si>
+    <t>bbbbb</t>
   </si>
   <si>
     <t>ARAUJO ROJAS, RICARDO ALEXANDER</t>
@@ -2666,43 +2672,45 @@
       <c r="A10" s="86">
         <v>1</v>
       </c>
-      <c r="B10" s="87"/>
+      <c r="B10" s="87" t="s">
+        <v>38</v>
+      </c>
       <c r="C10" s="88" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D10" s="89" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="90">
-        <v>10</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="E10" s="90"/>
       <c r="F10" s="91">
         <f>E10*35%</f>
       </c>
-      <c r="G10" s="90">
-        <v>10</v>
-      </c>
+      <c r="G10" s="90"/>
       <c r="H10" s="92">
         <f>G10*35%</f>
       </c>
-      <c r="I10" s="90">
-        <v>6</v>
-      </c>
+      <c r="I10" s="90"/>
       <c r="J10" s="93">
         <f>I10*30%</f>
       </c>
       <c r="K10" s="94">
         <f>ROUND((F10+H10+J10),2)</f>
       </c>
-      <c r="L10" s="90"/>
+      <c r="L10" s="90">
+        <v>10</v>
+      </c>
       <c r="M10" s="92">
         <f>L10*35%</f>
       </c>
-      <c r="N10" s="90"/>
+      <c r="N10" s="90">
+        <v>10</v>
+      </c>
       <c r="O10" s="92">
         <f>N10*35%</f>
       </c>
-      <c r="P10" s="90"/>
+      <c r="P10" s="90">
+        <v>6</v>
+      </c>
       <c r="Q10" s="93">
         <f>P10*30%</f>
       </c>
@@ -2755,43 +2763,45 @@
       <c r="A11" s="98">
         <v>2</v>
       </c>
-      <c r="B11" s="87"/>
+      <c r="B11" s="87" t="s">
+        <v>41</v>
+      </c>
       <c r="C11" s="88" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D11" s="89" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" s="99">
-        <v>8</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="E11" s="99"/>
       <c r="F11" s="100">
         <f>E11*35%</f>
       </c>
-      <c r="G11" s="99">
-        <v>8</v>
-      </c>
+      <c r="G11" s="99"/>
       <c r="H11" s="101">
         <f>G11*35%</f>
       </c>
-      <c r="I11" s="99">
-        <v>8</v>
-      </c>
+      <c r="I11" s="99"/>
       <c r="J11" s="102">
         <f>I11*30%</f>
       </c>
       <c r="K11" s="94">
         <f>ROUND((F11+H11+J11),2)</f>
       </c>
-      <c r="L11" s="99"/>
+      <c r="L11" s="99">
+        <v>8</v>
+      </c>
       <c r="M11" s="101">
         <f>L11*35%</f>
       </c>
-      <c r="N11" s="99"/>
+      <c r="N11" s="99">
+        <v>8</v>
+      </c>
       <c r="O11" s="101">
         <f>N11*35%</f>
       </c>
-      <c r="P11" s="99"/>
+      <c r="P11" s="99">
+        <v>8</v>
+      </c>
       <c r="Q11" s="102">
         <f>P11*30%</f>
       </c>
@@ -3067,7 +3077,7 @@
       <c r="B12" s="87"/>
       <c r="C12" s="88"/>
       <c r="D12" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E12" s="90"/>
       <c r="F12" s="100">
@@ -3148,7 +3158,7 @@
       <c r="B13" s="87"/>
       <c r="C13" s="88"/>
       <c r="D13" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E13" s="90"/>
       <c r="F13" s="100">
@@ -3229,7 +3239,7 @@
       <c r="B14" s="87"/>
       <c r="C14" s="88"/>
       <c r="D14" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E14" s="90"/>
       <c r="F14" s="100">
@@ -3310,7 +3320,7 @@
       <c r="B15" s="87"/>
       <c r="C15" s="88"/>
       <c r="D15" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E15" s="90"/>
       <c r="F15" s="100">
@@ -3391,7 +3401,7 @@
       <c r="B16" s="87"/>
       <c r="C16" s="88"/>
       <c r="D16" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E16" s="90"/>
       <c r="F16" s="100">
@@ -3472,7 +3482,7 @@
       <c r="B17" s="87"/>
       <c r="C17" s="88"/>
       <c r="D17" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E17" s="90"/>
       <c r="F17" s="100">
@@ -3553,7 +3563,7 @@
       <c r="B18" s="87"/>
       <c r="C18" s="88"/>
       <c r="D18" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E18" s="90"/>
       <c r="F18" s="100">
@@ -3635,7 +3645,7 @@
       <c r="B19" s="87"/>
       <c r="C19" s="88"/>
       <c r="D19" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E19" s="90"/>
       <c r="F19" s="100">
@@ -3717,7 +3727,7 @@
       <c r="B20" s="87"/>
       <c r="C20" s="88"/>
       <c r="D20" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E20" s="90"/>
       <c r="F20" s="100">
@@ -3799,7 +3809,7 @@
       <c r="B21" s="87"/>
       <c r="C21" s="88"/>
       <c r="D21" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E21" s="90"/>
       <c r="F21" s="100">
@@ -3881,7 +3891,7 @@
       <c r="B22" s="87"/>
       <c r="C22" s="88"/>
       <c r="D22" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E22" s="90"/>
       <c r="F22" s="100">
@@ -3963,7 +3973,7 @@
       <c r="B23" s="87"/>
       <c r="C23" s="88"/>
       <c r="D23" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E23" s="90"/>
       <c r="F23" s="100">
@@ -4045,7 +4055,7 @@
       <c r="B24" s="87"/>
       <c r="C24" s="88"/>
       <c r="D24" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E24" s="90"/>
       <c r="F24" s="100">
@@ -4127,7 +4137,7 @@
       <c r="B25" s="87"/>
       <c r="C25" s="88"/>
       <c r="D25" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E25" s="90"/>
       <c r="F25" s="100">
@@ -4209,7 +4219,7 @@
       <c r="B26" s="87"/>
       <c r="C26" s="88"/>
       <c r="D26" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E26" s="90"/>
       <c r="F26" s="100">
@@ -4291,7 +4301,7 @@
       <c r="B27" s="87"/>
       <c r="C27" s="88"/>
       <c r="D27" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E27" s="90"/>
       <c r="F27" s="100">
@@ -4373,7 +4383,7 @@
       <c r="B28" s="87"/>
       <c r="C28" s="88"/>
       <c r="D28" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E28" s="90"/>
       <c r="F28" s="100">
@@ -4455,7 +4465,7 @@
       <c r="B29" s="87"/>
       <c r="C29" s="88"/>
       <c r="D29" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E29" s="90"/>
       <c r="F29" s="100">
@@ -4537,7 +4547,7 @@
       <c r="B30" s="87"/>
       <c r="C30" s="88"/>
       <c r="D30" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E30" s="90"/>
       <c r="F30" s="100">
@@ -4619,7 +4629,7 @@
       <c r="B31" s="87"/>
       <c r="C31" s="88"/>
       <c r="D31" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E31" s="90"/>
       <c r="F31" s="100">
@@ -4701,7 +4711,7 @@
       <c r="B32" s="87"/>
       <c r="C32" s="88"/>
       <c r="D32" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E32" s="90"/>
       <c r="F32" s="100">
@@ -4783,7 +4793,7 @@
       <c r="B33" s="87"/>
       <c r="C33" s="88"/>
       <c r="D33" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E33" s="106"/>
       <c r="F33" s="100">
@@ -4865,7 +4875,7 @@
       <c r="B34" s="87"/>
       <c r="C34" s="88"/>
       <c r="D34" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E34" s="90"/>
       <c r="F34" s="100">
@@ -4939,7 +4949,7 @@
       </c>
       <c r="AK34" s="110"/>
       <c r="AL34" s="111" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -4949,7 +4959,7 @@
       <c r="B35" s="87"/>
       <c r="C35" s="88"/>
       <c r="D35" s="89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E35" s="90"/>
       <c r="F35" s="100">
@@ -5023,7 +5033,7 @@
       </c>
       <c r="AK35" s="112"/>
       <c r="AL35" s="113" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -5033,7 +5043,7 @@
       <c r="B36" s="87"/>
       <c r="C36" s="88"/>
       <c r="D36" s="89" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E36" s="90"/>
       <c r="F36" s="100">
@@ -5107,7 +5117,7 @@
       </c>
       <c r="AK36" s="112"/>
       <c r="AL36" s="113" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -5189,7 +5199,7 @@
       </c>
       <c r="AK37" s="112"/>
       <c r="AL37" s="113" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -5271,7 +5281,7 @@
       </c>
       <c r="AK38" s="112"/>
       <c r="AL38" s="113" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -5353,7 +5363,7 @@
       </c>
       <c r="AK39" s="112"/>
       <c r="AL39" s="114" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" ht="14.25" customHeight="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -7361,31 +7371,31 @@
     <row r="67" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="68" ht="14.25" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C68" s="139" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D68" s="1"/>
       <c r="E68" s="140"/>
       <c r="F68" s="141" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G68" s="142"/>
       <c r="H68" s="141" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I68" s="142"/>
       <c r="J68" s="141" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K68" s="141" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M68" s="143" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="69" ht="13.5" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C69" s="144" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D69" s="1"/>
       <c r="E69" s="145"/>
@@ -7409,7 +7419,7 @@
     </row>
     <row r="70" ht="12.75" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C70" s="148" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D70" s="1"/>
       <c r="E70" s="149"/>
@@ -7433,7 +7443,7 @@
     </row>
     <row r="71" ht="12.75" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C71" s="148" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="149"/>
@@ -7457,7 +7467,7 @@
     </row>
     <row r="72" ht="12.75" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C72" s="148" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="149"/>
@@ -7481,7 +7491,7 @@
     </row>
     <row r="73" ht="12.75" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C73" s="148" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D73" s="1"/>
       <c r="E73" s="149"/>
@@ -7505,7 +7515,7 @@
     </row>
     <row r="74" ht="12.75" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C74" s="148" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="149"/>
@@ -7529,7 +7539,7 @@
     </row>
     <row r="75" ht="13.5" customHeight="1" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C75" s="153" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D75" s="1"/>
       <c r="E75" s="154"/>
@@ -7779,28 +7789,28 @@
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="157" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" s="158" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="159" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D1" s="159" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="159" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="157" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G1" s="157" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H1" s="157" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9307,7 +9317,7 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="161" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="161"/>
       <c r="C1" s="161"/>
@@ -9333,7 +9343,7 @@
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="161" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B2" s="161"/>
       <c r="C2" s="161"/>
@@ -9359,14 +9369,14 @@
     </row>
     <row r="3" ht="12.75" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="163" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="163"/>
       <c r="C3" s="163"/>
       <c r="D3" s="163"/>
       <c r="E3" s="163"/>
       <c r="F3" s="163" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G3" s="163"/>
       <c r="H3" s="163"/>
@@ -9375,7 +9385,7 @@
       <c r="K3" s="163"/>
       <c r="L3" s="163"/>
       <c r="M3" s="164" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N3" s="165">
         <v>2026</v>
@@ -9391,7 +9401,7 @@
     </row>
     <row r="4" ht="12.75" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="166" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" s="166"/>
       <c r="C4" s="166"/>
@@ -9408,7 +9418,7 @@
       </c>
       <c r="M4" s="163"/>
       <c r="N4" s="168" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O4" s="163"/>
       <c r="P4" s="163"/>
@@ -9421,12 +9431,12 @@
     </row>
     <row r="5" ht="12.75" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="166" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" s="166"/>
       <c r="C5" s="166"/>
       <c r="D5" s="167" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E5" s="167"/>
       <c r="F5" s="167"/>
@@ -9449,7 +9459,7 @@
     </row>
     <row r="6" ht="13.5" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="169" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B6" s="169"/>
       <c r="C6" s="169"/>
@@ -9464,7 +9474,7 @@
       <c r="L6" s="170"/>
       <c r="M6" s="170"/>
       <c r="N6" s="164" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O6" s="163"/>
       <c r="P6" s="163"/>
@@ -9477,7 +9487,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="172" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="173" t="s">
         <v>23</v>
@@ -9486,35 +9496,35 @@
         <v>24</v>
       </c>
       <c r="D7" s="174" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E7" s="175" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F7" s="175"/>
       <c r="G7" s="175"/>
       <c r="H7" s="175"/>
       <c r="I7" s="175"/>
       <c r="J7" s="175" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K7" s="175"/>
       <c r="L7" s="175"/>
       <c r="M7" s="175"/>
       <c r="N7" s="175"/>
       <c r="O7" s="176" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="P7" s="176"/>
       <c r="Q7" s="176"/>
       <c r="R7" s="176"/>
       <c r="S7" s="176"/>
       <c r="T7" s="177" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="U7" s="177"/>
       <c r="V7" s="178" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" ht="65.25" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -9523,55 +9533,55 @@
       <c r="C8" s="172"/>
       <c r="D8" s="174"/>
       <c r="E8" s="179" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F8" s="179" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="179" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="179" t="s">
         <v>87</v>
-      </c>
-      <c r="G8" s="179" t="s">
-        <v>88</v>
-      </c>
-      <c r="H8" s="179" t="s">
-        <v>85</v>
       </c>
       <c r="I8" s="180">
         <v>0.25</v>
       </c>
       <c r="J8" s="179" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K8" s="179" t="s">
+        <v>89</v>
+      </c>
+      <c r="L8" s="179" t="s">
+        <v>90</v>
+      </c>
+      <c r="M8" s="179" t="s">
         <v>87</v>
-      </c>
-      <c r="L8" s="179" t="s">
-        <v>88</v>
-      </c>
-      <c r="M8" s="179" t="s">
-        <v>85</v>
       </c>
       <c r="N8" s="180">
         <v>0.5</v>
       </c>
       <c r="O8" s="179" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="P8" s="179" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q8" s="179" t="s">
+        <v>90</v>
+      </c>
+      <c r="R8" s="179" t="s">
         <v>87</v>
-      </c>
-      <c r="Q8" s="179" t="s">
-        <v>88</v>
-      </c>
-      <c r="R8" s="179" t="s">
-        <v>85</v>
       </c>
       <c r="S8" s="180">
         <v>0.25</v>
       </c>
       <c r="T8" s="181" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="U8" s="182" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="V8" s="178"/>
     </row>
@@ -9583,10 +9593,10 @@
         <v>19770108</v>
       </c>
       <c r="C9" s="185" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E9" s="187"/>
       <c r="F9" s="187"/>
@@ -9639,10 +9649,10 @@
         <v>3669191</v>
       </c>
       <c r="C10" s="185" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D10" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E10" s="187"/>
       <c r="F10" s="187"/>
@@ -9695,10 +9705,10 @@
         <v>19913116</v>
       </c>
       <c r="C11" s="185" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D11" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E11" s="187"/>
       <c r="F11" s="187"/>
@@ -9751,10 +9761,10 @@
         <v>19769700</v>
       </c>
       <c r="C12" s="185" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D12" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12" s="187"/>
       <c r="F12" s="187"/>
@@ -9807,10 +9817,10 @@
         <v>19769732</v>
       </c>
       <c r="C13" s="185" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D13" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E13" s="187"/>
       <c r="F13" s="187"/>
@@ -9863,10 +9873,10 @@
         <v>19769682</v>
       </c>
       <c r="C14" s="185" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E14" s="187"/>
       <c r="F14" s="187"/>
@@ -9919,10 +9929,10 @@
         <v>19913170</v>
       </c>
       <c r="C15" s="185" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D15" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E15" s="187"/>
       <c r="F15" s="187"/>
@@ -9975,10 +9985,10 @@
         <v>5059703</v>
       </c>
       <c r="C16" s="185" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D16" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E16" s="187"/>
       <c r="F16" s="187"/>
@@ -10031,10 +10041,10 @@
         <v>19770269</v>
       </c>
       <c r="C17" s="185" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D17" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E17" s="187"/>
       <c r="F17" s="187"/>
@@ -10087,10 +10097,10 @@
         <v>20238015</v>
       </c>
       <c r="C18" s="185" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D18" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E18" s="187"/>
       <c r="F18" s="187"/>
@@ -10143,10 +10153,10 @@
         <v>19846395</v>
       </c>
       <c r="C19" s="185" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D19" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E19" s="187"/>
       <c r="F19" s="187"/>
@@ -10199,10 +10209,10 @@
         <v>19913145</v>
       </c>
       <c r="C20" s="185" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D20" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E20" s="187"/>
       <c r="F20" s="187"/>
@@ -10255,10 +10265,10 @@
         <v>19769931</v>
       </c>
       <c r="C21" s="185" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D21" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E21" s="187"/>
       <c r="F21" s="187"/>
@@ -10311,10 +10321,10 @@
         <v>3669150</v>
       </c>
       <c r="C22" s="185" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D22" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E22" s="187"/>
       <c r="F22" s="187"/>
@@ -10367,10 +10377,10 @@
         <v>19913258</v>
       </c>
       <c r="C23" s="185" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D23" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E23" s="187"/>
       <c r="F23" s="187"/>
@@ -10423,10 +10433,10 @@
         <v>3669163</v>
       </c>
       <c r="C24" s="185" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D24" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E24" s="187"/>
       <c r="F24" s="187"/>
@@ -10479,10 +10489,10 @@
         <v>19770150</v>
       </c>
       <c r="C25" s="185" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D25" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E25" s="187"/>
       <c r="F25" s="187"/>
@@ -10535,10 +10545,10 @@
         <v>19913305</v>
       </c>
       <c r="C26" s="185" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D26" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E26" s="187"/>
       <c r="F26" s="187"/>
@@ -10591,10 +10601,10 @@
         <v>19983921</v>
       </c>
       <c r="C27" s="185" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D27" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E27" s="187"/>
       <c r="F27" s="187"/>
@@ -10647,10 +10657,10 @@
         <v>19770274</v>
       </c>
       <c r="C28" s="185" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D28" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E28" s="187"/>
       <c r="F28" s="187"/>
@@ -10703,10 +10713,10 @@
         <v>19769851</v>
       </c>
       <c r="C29" s="185" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D29" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E29" s="187"/>
       <c r="F29" s="187"/>
@@ -10759,10 +10769,10 @@
         <v>19913310</v>
       </c>
       <c r="C30" s="185" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D30" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E30" s="187"/>
       <c r="F30" s="187"/>
@@ -10815,10 +10825,10 @@
         <v>19769690</v>
       </c>
       <c r="C31" s="185" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D31" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E31" s="187"/>
       <c r="F31" s="187"/>
@@ -10871,10 +10881,10 @@
         <v>19770293</v>
       </c>
       <c r="C32" s="185" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D32" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E32" s="187"/>
       <c r="F32" s="187"/>
@@ -10927,10 +10937,10 @@
         <v>20054579</v>
       </c>
       <c r="C33" s="185" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D33" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E33" s="187"/>
       <c r="F33" s="187"/>
@@ -10983,10 +10993,10 @@
         <v>19769691</v>
       </c>
       <c r="C34" s="185" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D34" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E34" s="187"/>
       <c r="F34" s="187"/>
@@ -11039,10 +11049,10 @@
         <v>19769956</v>
       </c>
       <c r="C35" s="185" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D35" s="186" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E35" s="187"/>
       <c r="F35" s="187"/>
@@ -11095,10 +11105,10 @@
         <v>19770033</v>
       </c>
       <c r="C36" s="185" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D36" s="186" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E36" s="187"/>
       <c r="F36" s="187"/>

</xml_diff>